<commit_message>
Update Track 1 methods form to 17-gene panel; add repo AGENTS.md + mva-hackathon skill.
Methods xlsx rows 9/19 now reflect SLF2/SMC5 (post-audit extension, verified
clean post-hoc). AGENTS.md + .agents/skills/mva-hackathon/ document the agent
contract used in this repo.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/submissions/Ryukijano_track1_methods.xlsx
+++ b/submissions/Ryukijano_track1_methods.xlsx
@@ -549,7 +549,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Ensembl VEP 116 (GRCh38, offline cache, AlphaMissense + popEVE/EVE plugins) -&gt; 15-gene mitotic/SAC panel filter (configs/panel.yaml) -&gt; rarity filter (gnomADg_AF, gnomADe_AF, AF all missing or &lt;=0.001) -&gt; consequence filter (stop_gained, missense, canonical splice, frameshift) -&gt; SpliceAI (-D 500 on the candidate VCF; -D 4999 deep sweep across chr15:40.18-40.30 Mb) -&gt; per-variant pathogenicity score (PTV 0.99; missense 0.7*popEVE_sigmoid + 0.3*AlphaMissense; splice-region max DS) -&gt; compound-het pair product -&gt; EPCR = max(0.95 floor, pair product). Only BUB1B carried two rare functional alleles: p.Leu737Ter (ClinVar P/LP, VCV000533901) + p.Asn1002Lys (AlphaMissense 0.9229; ClinVar VUS for the same protein change via c.3006T&gt;A, VCV004600147.1; exact c.3006T&gt;G absent from ClinVar, 1 gnomAD v4 exome allele). Post-hoc: AlphaGenome AVI (33.76 / 25.61 Phred), WhatsHap read-backed phasing on the 84 GB FASTQs (UNRESOLVED: 10.9 kb gap, one intervening het, ~1.3 kb max insert), ClinVar/gnomAD/dbSNP live re-verification.</t>
+          <t>Ensembl VEP 116 (GRCh38, offline cache, AlphaMissense + popEVE/EVE plugins) -&gt; 17-gene mitotic/SAC panel (SLF2/SMC5 Atelis genes added post-audit; post-hoc VEP check confirmed no causal variant in either) filter (configs/panel.yaml) -&gt; rarity filter (gnomADg_AF, gnomADe_AF, AF all missing or &lt;=0.001) -&gt; consequence filter (stop_gained, missense, canonical splice, frameshift) -&gt; SpliceAI (-D 500 on the candidate VCF; -D 4999 deep sweep across chr15:40.18-40.30 Mb) -&gt; per-variant pathogenicity score (PTV 0.99; missense 0.7*popEVE_sigmoid + 0.3*AlphaMissense; splice-region max DS) -&gt; compound-het pair product -&gt; EPCR = max(0.95 floor, pair product). Only BUB1B carried two rare functional alleles: p.Leu737Ter (ClinVar P/LP, VCV000533901) + p.Asn1002Lys (AlphaMissense 0.9229; ClinVar VUS for the same protein change via c.3006T&gt;A, VCV004600147.1; exact c.3006T&gt;G absent from ClinVar, 1 gnomAD v4 exome allele). Post-hoc: AlphaGenome AVI (33.76 / 25.61 Phred), WhatsHap read-backed phasing on the 84 GB FASTQs (UNRESOLVED: 10.9 kb gap, one intervening het, ~1.3 kb max insert), ClinVar/gnomAD/dbSNP live re-verification.</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>We filtered the gated WGS VCF through a 15-gene mitotic-checkpoint panel (BUB1B, BUB1, MAD1L1, TRIP13, MAD2L1BP, CEP57, CEP192, CENATAC, CDC20, TTK, MAD2L1, BUB3, KNL1, AURKA, PLK1) after Ensembl VEP 116 annotation with AlphaMissense and popEVE, keeping variants with all gnomAD AF fields &lt;=0.001 and functional consequences. Only BUB1B carried two rare functional alleles: p.Leu737Ter (ClinVar P/LP for MVA1) and p.Asn1002Lys (AlphaMissense 0.9229; same protein change is a single-submitter ClinVar VUS via c.3006T&gt;A). The architecture matches the canonical viable MVA1 pattern (truncating allele + hypomorphic C-lobe pseudokinase missense, Hanks 2004). We submitted one primary row at EPCR 0.95 (pair product ~0.91 floored to the primary floor). Strengths: reproducible CLI (scripts/run_track1.py), a local clone of the official scorer verified against the live Space evaluation.py, live ClinVar/gnomAD/dbSNP re-verification, a SpliceAI -D 4999 deep-intronic sweep closing the cryptic-splice falsifier, AlphaGenome AVI as a second in-silico layer, and honest pre-registered falsification tests (ESM-1v rejected N1002K-as-L1012P; PrimeKG rejected rapalog discovery). Limitations: read-backed phasing is UNRESOLVED (the 10.9 kb gap is unbridgeable by 150 bp PE reads and only one intervening het SNV exists); compound heterozygosity is therefore inferred from MVA1 architecture and absence of competing candidates, not molecularly proven; N1002K has no direct functional assay and predictors conflict (AlphaMissense pathogenic vs ESM-1v mild); short-read WGS cannot fully exclude a deep-intronic/regulatory/Alu-SVA second hit (a documented MVA1 mechanism); residual BUBR1 (11%+/-3%) is a mouse literature value, not measured in this child. Parental genotyping or long-range PCR + long-read sequencing would definitively resolve phase.</t>
+          <t>We filtered the gated WGS VCF through a 17-gene mitotic-checkpoint panel (incl. SLF2/SMC5 Atelis genes, verified clean post-hoc) (BUB1B, BUB1, MAD1L1, TRIP13, MAD2L1BP, CEP57, CEP192, CENATAC, SLF2, SMC5, CDC20, TTK, MAD2L1, BUB3, KNL1, AURKA, PLK1) after Ensembl VEP 116 annotation with AlphaMissense and popEVE, keeping variants with all gnomAD AF fields &lt;=0.001 and functional consequences. Only BUB1B carried two rare functional alleles: p.Leu737Ter (ClinVar P/LP for MVA1) and p.Asn1002Lys (AlphaMissense 0.9229; same protein change is a single-submitter ClinVar VUS via c.3006T&gt;A). The architecture matches the canonical viable MVA1 pattern (truncating allele + hypomorphic C-lobe pseudokinase missense, Hanks 2004). We submitted one primary row at EPCR 0.95 (pair product ~0.91 floored to the primary floor). Strengths: reproducible CLI (scripts/run_track1.py), a local clone of the official scorer verified against the live Space evaluation.py, live ClinVar/gnomAD/dbSNP re-verification, a SpliceAI -D 4999 deep-intronic sweep closing the cryptic-splice falsifier, AlphaGenome AVI as a second in-silico layer, and honest pre-registered falsification tests (ESM-1v rejected N1002K-as-L1012P; PrimeKG rejected rapalog discovery). Limitations: read-backed phasing is UNRESOLVED (the 10.9 kb gap is unbridgeable by 150 bp PE reads and only one intervening het SNV exists); compound heterozygosity is therefore inferred from MVA1 architecture and absence of competing candidates, not molecularly proven; N1002K has no direct functional assay and predictors conflict (AlphaMissense pathogenic vs ESM-1v mild); short-read WGS cannot fully exclude a deep-intronic/regulatory/Alu-SVA second hit (a documented MVA1 mechanism); residual BUBR1 (11%+/-3%) is a mouse literature value, not measured in this child. Parental genotyping or long-range PCR + long-read sequencing would definitively resolve phase.</t>
         </is>
       </c>
     </row>

</xml_diff>